<commit_message>
Finnished version - few small tweaks remaining
</commit_message>
<xml_diff>
--- a/SW/DISPLAY SCREENS.xlsx
+++ b/SW/DISPLAY SCREENS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://schaeffler-my.sharepoint.com/personal/uiv10467_vitesco_com/Documents/Plocha/automatedelectrictestingsystem_aets/SW/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://schaeffler-my.sharepoint.com/personal/uiv10467_vitesco_com/Documents/Plocha/AETS/AETS/SW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1233" documentId="8_{D1488593-6CCD-4D42-B221-91528AA5051D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{22A6D618-77F3-44F2-B890-371D6D92AD2F}"/>
+  <xr:revisionPtr revIDLastSave="1300" documentId="8_{D1488593-6CCD-4D42-B221-91528AA5051D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9188476F-3406-40C3-B8DE-87E53B68FE8A}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E6C8F8F3-ACBD-40E2-94DA-A7435C16BF12}"/>
+    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" activeTab="1" xr2:uid="{E6C8F8F3-ACBD-40E2-94DA-A7435C16BF12}"/>
   </bookViews>
   <sheets>
     <sheet name="Templates" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1754" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="86">
   <si>
     <t>A</t>
   </si>
@@ -290,6 +290,12 @@
   <si>
     <t>TEST OK</t>
   </si>
+  <si>
+    <t>RELAY COUNT LOW</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
 </sst>
 </file>
 
@@ -412,7 +418,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -452,6 +458,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1880,6 +1889,112 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>77</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>80</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="2" name="Straight Arrow Connector 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A3D6DBE-BE77-4FB2-A842-CCCFBCD18FAD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="48539400" y="5867400"/>
+          <a:ext cx="2324100" cy="3314700"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="152400">
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>91</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>91</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="7" name="Straight Arrow Connector 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2F2E205-78D6-4193-AEA7-07C33D96813C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="59016900" y="1485900"/>
+          <a:ext cx="0" cy="2057400"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="152400">
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2200,7 +2315,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{497F4F3F-DF2C-4A2F-A59B-E650E6ED4318}">
-  <dimension ref="B3:AV117"/>
+  <dimension ref="B3:AV123"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="24.5703125" customWidth="1"/>
@@ -6873,37 +6988,227 @@
       <c r="W117" s="1"/>
       <c r="X117" s="1"/>
     </row>
+    <row r="119" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="120" spans="2:24" ht="32.25" x14ac:dyDescent="0.25">
+      <c r="B120" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C120" s="3"/>
+      <c r="E120" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F120" s="1"/>
+      <c r="G120" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H120" s="1"/>
+      <c r="I120" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J120" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K120" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L120" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M120" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N120" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="O120" s="1"/>
+      <c r="P120" s="1"/>
+      <c r="Q120" s="1"/>
+      <c r="R120" s="1"/>
+      <c r="S120" s="1"/>
+      <c r="T120" s="1"/>
+      <c r="U120" s="1"/>
+      <c r="V120" s="1"/>
+      <c r="W120" s="1"/>
+      <c r="X120" s="1"/>
+    </row>
+    <row r="121" spans="2:24" ht="32.25" x14ac:dyDescent="0.25">
+      <c r="B121" s="4"/>
+      <c r="C121" s="5"/>
+      <c r="E121" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G121" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H121" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="I121" s="1"/>
+      <c r="J121" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="K121" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L121" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="M121" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N121" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="O121" s="1"/>
+      <c r="P121" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q121" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="R121" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="S121" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="T121" s="1"/>
+      <c r="U121" s="1"/>
+      <c r="V121" s="1"/>
+      <c r="W121" s="1"/>
+      <c r="X121" s="1"/>
+    </row>
+    <row r="122" spans="2:24" ht="32.25" x14ac:dyDescent="0.25">
+      <c r="B122" s="4"/>
+      <c r="C122" s="5"/>
+      <c r="E122" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G122" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J122" s="1"/>
+      <c r="K122" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="L122" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="M122" s="1"/>
+      <c r="N122" s="1"/>
+      <c r="O122" s="1"/>
+      <c r="P122" s="1"/>
+      <c r="Q122" s="1"/>
+      <c r="R122" s="1"/>
+      <c r="S122" s="1"/>
+      <c r="T122" s="1"/>
+      <c r="U122" s="1"/>
+      <c r="V122" s="1"/>
+      <c r="W122" s="1"/>
+      <c r="X122" s="1"/>
+    </row>
+    <row r="123" spans="2:24" ht="33" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B123" s="6"/>
+      <c r="C123" s="7"/>
+      <c r="E123" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G123" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H123" s="1"/>
+      <c r="I123" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J123" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K123" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L123" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M123" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="N123" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="O123" s="1"/>
+      <c r="P123" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q123" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="R123" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="S123" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="T123" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="U123" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="V123" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W123" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="X123" s="1"/>
+    </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="B96:C99"/>
-    <mergeCell ref="B108:C111"/>
-    <mergeCell ref="B102:C105"/>
-    <mergeCell ref="B114:C117"/>
-    <mergeCell ref="Z86:AA89"/>
-    <mergeCell ref="Z74:AA77"/>
-    <mergeCell ref="Z57:AA60"/>
-    <mergeCell ref="Z62:AA65"/>
-    <mergeCell ref="Z69:AA72"/>
-    <mergeCell ref="B80:C83"/>
-    <mergeCell ref="B86:C89"/>
-    <mergeCell ref="B73:C76"/>
-    <mergeCell ref="Z27:AA30"/>
-    <mergeCell ref="Z32:AA35"/>
-    <mergeCell ref="Z37:AA40"/>
-    <mergeCell ref="Z43:AA46"/>
-    <mergeCell ref="Z79:AA82"/>
-    <mergeCell ref="B42:C45"/>
-    <mergeCell ref="B47:C50"/>
-    <mergeCell ref="B52:C55"/>
-    <mergeCell ref="B57:C60"/>
-    <mergeCell ref="B62:C65"/>
-    <mergeCell ref="B68:C71"/>
+  <mergeCells count="30">
+    <mergeCell ref="B120:C123"/>
     <mergeCell ref="B4:C7"/>
     <mergeCell ref="B9:C12"/>
     <mergeCell ref="B27:C30"/>
     <mergeCell ref="Z49:AA52"/>
     <mergeCell ref="B14:C17"/>
     <mergeCell ref="B32:C35"/>
+    <mergeCell ref="B42:C45"/>
+    <mergeCell ref="B47:C50"/>
+    <mergeCell ref="B52:C55"/>
+    <mergeCell ref="B57:C60"/>
+    <mergeCell ref="B62:C65"/>
+    <mergeCell ref="Z27:AA30"/>
+    <mergeCell ref="Z32:AA35"/>
+    <mergeCell ref="Z37:AA40"/>
+    <mergeCell ref="Z43:AA46"/>
+    <mergeCell ref="Z79:AA82"/>
+    <mergeCell ref="Z74:AA77"/>
+    <mergeCell ref="Z57:AA60"/>
+    <mergeCell ref="Z62:AA65"/>
+    <mergeCell ref="Z69:AA72"/>
+    <mergeCell ref="B80:C83"/>
+    <mergeCell ref="B73:C76"/>
+    <mergeCell ref="B68:C71"/>
+    <mergeCell ref="B96:C99"/>
+    <mergeCell ref="B108:C111"/>
+    <mergeCell ref="B102:C105"/>
+    <mergeCell ref="B114:C117"/>
+    <mergeCell ref="Z86:AA89"/>
+    <mergeCell ref="B86:C89"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -6977,7 +7282,7 @@
       <c r="DZ17" s="1"/>
       <c r="EA17" s="1"/>
     </row>
-    <row r="18" spans="82:131" ht="32.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="82:131" ht="33" thickBot="1" x14ac:dyDescent="0.3">
       <c r="DE18" s="4"/>
       <c r="DF18" s="5"/>
       <c r="DH18" s="1"/>
@@ -7024,6 +7329,46 @@
       <c r="EA18" s="1"/>
     </row>
     <row r="19" spans="82:131" ht="32.25" x14ac:dyDescent="0.25">
+      <c r="CD19" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="CE19" s="3"/>
+      <c r="CG19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="CH19" s="1"/>
+      <c r="CI19" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="CJ19" s="1"/>
+      <c r="CK19" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="CL19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="CM19" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="CN19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="CO19" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="CP19" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="CQ19" s="1"/>
+      <c r="CR19" s="1"/>
+      <c r="CS19" s="1"/>
+      <c r="CT19" s="1"/>
+      <c r="CU19" s="1"/>
+      <c r="CV19" s="1"/>
+      <c r="CW19" s="1"/>
+      <c r="CX19" s="1"/>
+      <c r="CY19" s="1"/>
+      <c r="CZ19" s="1"/>
       <c r="DE19" s="4"/>
       <c r="DF19" s="5"/>
       <c r="DH19" s="1"/>
@@ -7048,6 +7393,54 @@
       <c r="EA19" s="1"/>
     </row>
     <row r="20" spans="82:131" ht="33" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="CD20" s="4"/>
+      <c r="CE20" s="5"/>
+      <c r="CG20" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="CH20" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="CI20" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="CJ20" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="CK20" s="1"/>
+      <c r="CL20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="CM20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="CN20" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="CO20" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="CP20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="CQ20" s="1"/>
+      <c r="CR20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="CS20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="CT20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="CU20" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="CV20" s="1"/>
+      <c r="CW20" s="1"/>
+      <c r="CX20" s="1"/>
+      <c r="CY20" s="1"/>
+      <c r="CZ20" s="1"/>
       <c r="DE20" s="6"/>
       <c r="DF20" s="7"/>
       <c r="DH20" s="1"/>
@@ -7071,7 +7464,102 @@
       <c r="DZ20" s="1"/>
       <c r="EA20" s="1"/>
     </row>
-    <row r="22" spans="82:131" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="21" spans="82:131" ht="32.25" x14ac:dyDescent="0.25">
+      <c r="CD21" s="4"/>
+      <c r="CE21" s="5"/>
+      <c r="CG21" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="CH21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="CI21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="CJ21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="CK21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="CL21" s="1"/>
+      <c r="CM21" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="CN21" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="CO21" s="1"/>
+      <c r="CP21" s="1"/>
+      <c r="CQ21" s="1"/>
+      <c r="CR21" s="1"/>
+      <c r="CS21" s="1"/>
+      <c r="CT21" s="1"/>
+      <c r="CU21" s="1"/>
+      <c r="CV21" s="1"/>
+      <c r="CW21" s="1"/>
+      <c r="CX21" s="1"/>
+      <c r="CY21" s="1"/>
+      <c r="CZ21" s="1"/>
+    </row>
+    <row r="22" spans="82:131" ht="33" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="CD22" s="6"/>
+      <c r="CE22" s="7"/>
+      <c r="CG22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="CH22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="CI22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="CJ22" s="1"/>
+      <c r="CK22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="CL22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="CM22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="CN22" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="CO22" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="CP22" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="CQ22" s="1"/>
+      <c r="CR22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="CS22" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="CT22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="CU22" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="CV22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="CW22" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="CX22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="CY22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="CZ22" s="1"/>
+    </row>
     <row r="23" spans="82:131" ht="32.25" x14ac:dyDescent="0.25">
       <c r="DE23" s="8" t="s">
         <v>83</v>
@@ -11579,7 +12067,21 @@
       <c r="BY130" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
+    <mergeCell ref="BC34:BD37"/>
+    <mergeCell ref="BC39:BD42"/>
+    <mergeCell ref="BC55:BD58"/>
+    <mergeCell ref="CD19:CE22"/>
+    <mergeCell ref="DE46:DF49"/>
+    <mergeCell ref="DE51:DF54"/>
+    <mergeCell ref="B67:C70"/>
+    <mergeCell ref="AB64:AC67"/>
+    <mergeCell ref="AB69:AC72"/>
+    <mergeCell ref="CD71:CE74"/>
+    <mergeCell ref="CD76:CE79"/>
+    <mergeCell ref="BC74:BD77"/>
+    <mergeCell ref="CD46:CE49"/>
+    <mergeCell ref="CD51:CE54"/>
     <mergeCell ref="BC127:BD130"/>
     <mergeCell ref="CD28:CE31"/>
     <mergeCell ref="CD34:CE37"/>
@@ -11596,19 +12098,6 @@
     <mergeCell ref="CD59:CE62"/>
     <mergeCell ref="CD64:CE67"/>
     <mergeCell ref="BC68:BD71"/>
-    <mergeCell ref="CD71:CE74"/>
-    <mergeCell ref="CD76:CE79"/>
-    <mergeCell ref="BC74:BD77"/>
-    <mergeCell ref="CD46:CE49"/>
-    <mergeCell ref="CD51:CE54"/>
-    <mergeCell ref="DE46:DF49"/>
-    <mergeCell ref="DE51:DF54"/>
-    <mergeCell ref="B67:C70"/>
-    <mergeCell ref="AB64:AC67"/>
-    <mergeCell ref="AB69:AC72"/>
-    <mergeCell ref="BC34:BD37"/>
-    <mergeCell ref="BC39:BD42"/>
-    <mergeCell ref="BC55:BD58"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>